<commit_message>
edit colour game Q and disyllable prac display
</commit_message>
<xml_diff>
--- a/epepep_structure.xlsx
+++ b/epepep_structure.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\annwa\OneDrive\Desktop\Workspace\epepep\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57D253D9-CE5E-4BAF-8665-1B0AA6385EE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F87FBE7-17B2-4CDC-A447-94E6A3290433}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="12863" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Word" sheetId="2" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1222" uniqueCount="746">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1270" uniqueCount="795">
   <si>
     <t>Unit</t>
   </si>
@@ -1466,9 +1466,6 @@
     <t>sei3 wai4</t>
   </si>
   <si>
-    <t>個案|照顧|聖誕|貢獻|更加|降低|背景|禁止|鏡頭|四圍|觀眾|關注|酒店|廣吿|投訴|門票</t>
-  </si>
-  <si>
     <t>大</t>
   </si>
   <si>
@@ -1815,9 +1812,6 @@
   </si>
   <si>
     <t>mou4 haan6</t>
-  </si>
-  <si>
-    <t>運動|任務|混亂|誤會|健康|第三|代表|系統|甚至|受到|例如|調查|關係|經驗|改善|總共|透露|訓練|成立|無限|</t>
   </si>
   <si>
     <t>Colour_colour</t>
@@ -1851,9 +1845,6 @@
     <t>他他提工工工工完工他完半半工他完提他制制半制他他提制半半制半半他工他工工講工提工工提他他講工提工工完工講講完工他工他他工他完工他</t>
   </si>
   <si>
-    <t>#e0e0e0,#808080,#9900ff,#ffffff</t>
-  </si>
-  <si>
     <t>#D5FDFF,#a4c2f4,#93E8FF,#1155cc,,#FFF4D1</t>
   </si>
   <si>
@@ -1896,9 +1887,6 @@
     <t>maa5</t>
   </si>
   <si>
-    <t>網</t>
-  </si>
-  <si>
     <t>mong5</t>
   </si>
   <si>
@@ -1941,12 +1929,6 @@
     <t>jan5</t>
   </si>
   <si>
-    <t>米</t>
-  </si>
-  <si>
-    <t>mai5</t>
-  </si>
-  <si>
     <t>遠</t>
   </si>
   <si>
@@ -1996,9 +1978,6 @@
   </si>
   <si>
     <t>勇</t>
-  </si>
-  <si>
-    <t>jung5</t>
   </si>
   <si>
     <t>染</t>
@@ -2058,9 +2037,6 @@
 第六調: #FFFFFF</t>
   </si>
   <si>
-    <t>奶!眼米</t>
-  </si>
-  <si>
     <t>螞蟻</t>
   </si>
   <si>
@@ -2070,9 +2046,6 @@
     <t>武</t>
   </si>
   <si>
-    <t>美理晚武也每引遠滿朗</t>
-  </si>
-  <si>
     <t>母語</t>
   </si>
   <si>
@@ -2094,9 +2067,6 @@
     <t>maa5 mei5</t>
   </si>
   <si>
-    <t>勇何染第件笑權</t>
-  </si>
-  <si>
     <t>領先</t>
   </si>
   <si>
@@ -2224,9 +2194,6 @@
   </si>
   <si>
     <t>!神免署永</t>
-  </si>
-  <si>
-    <t>勇勇勇勇勇染染染染染何何何權勇染勇權件笑笑第何染權第件笑笑件件權染權第笑笑第何勇勇勇何權權何染染染染勇勇勇勇染染勇染染染勇勇勇勇</t>
   </si>
   <si>
     <t>,,#864300,#525252,#FFF3E2,#FFFFFF</t>
@@ -2263,18 +2230,12 @@
     <t>miu5</t>
   </si>
   <si>
-    <t>秒我你腦買碼網與</t>
-  </si>
-  <si>
     <t>魯莽</t>
   </si>
   <si>
     <t>lou5 mong5</t>
   </si>
   <si>
-    <t>螞蟻|母語|魯莽|馬尾|領先|野豬|了解|敏感|挽救|軟化|儲存|偶然|冷淡|偉大|温暖|風雨|展覽|小鳥|快艇|器皿|行李|牛腩|伴舞|廟宇</t>
-  </si>
-  <si>
     <t>萬萬望望望萬萬望望投望望萬萬萬望聯投聯萬望望望投投瀉聯聯萬萬聯聯案瀉案投投投投案瀉品案瀉聯聯瀉品品班品案瀉瀉品品班班班品品品班班</t>
   </si>
   <si>
@@ -2294,6 +2255,192 @@
   </si>
   <si>
     <t>廣東話的第五調是低升調，調值為23。通常對應普通話第三聲（較多）､第四聲（較少）。</t>
+  </si>
+  <si>
+    <t>#e0e0e0,#808080,#9900ff,#ffffff,,</t>
+  </si>
+  <si>
+    <t>抗爭</t>
+  </si>
+  <si>
+    <t>kong3 zang1</t>
+  </si>
+  <si>
+    <t>破產</t>
+  </si>
+  <si>
+    <t>po3 caan2</t>
+  </si>
+  <si>
+    <t>肺炎</t>
+  </si>
+  <si>
+    <t>fai3 jim4</t>
+  </si>
+  <si>
+    <t>機構</t>
+  </si>
+  <si>
+    <t>gei1 kau3</t>
+  </si>
+  <si>
+    <t>口罩</t>
+  </si>
+  <si>
+    <t>hau2 zaau3</t>
+  </si>
+  <si>
+    <t>人數</t>
+  </si>
+  <si>
+    <t>jan4 sou3</t>
+  </si>
+  <si>
+    <t>個案|照顧|聖誕|貢獻|抗爭|更加|降低|背景|破產|禁止|鏡頭|四圍|肺炎|觀眾|機構|關注|酒店|廣吿|口罩|投訴|門票|人數</t>
+  </si>
+  <si>
+    <t>罷工</t>
+  </si>
+  <si>
+    <t>baa6 gung1</t>
+  </si>
+  <si>
+    <t>效果</t>
+  </si>
+  <si>
+    <t>haau6 gwo2</t>
+  </si>
+  <si>
+    <t>預計</t>
+  </si>
+  <si>
+    <t>jyu6 gai3</t>
+  </si>
+  <si>
+    <t>病人</t>
+  </si>
+  <si>
+    <t>beng6 jan4</t>
+  </si>
+  <si>
+    <t>方便</t>
+  </si>
+  <si>
+    <t>fong1 bin6</t>
+  </si>
+  <si>
+    <t>口號</t>
+  </si>
+  <si>
+    <t>hau2 hou6</t>
+  </si>
+  <si>
+    <t>破壞</t>
+  </si>
+  <si>
+    <t>po3 waai6</t>
+  </si>
+  <si>
+    <t>旗下</t>
+  </si>
+  <si>
+    <t>kei4 haa6</t>
+  </si>
+  <si>
+    <t>運動|任務|混亂|誤會|健康|第三|罷工|效果|代表|系統|甚至|受到|預計|病人|例如|調查|關係|方便|經驗|口號|改善|總共|透露|訓練|破壞|旗下|成立|無限|</t>
+  </si>
+  <si>
+    <t>有些</t>
+  </si>
+  <si>
+    <t>jau5 se1</t>
+  </si>
+  <si>
+    <t>妥</t>
+  </si>
+  <si>
+    <t>to5</t>
+  </si>
+  <si>
+    <t>勇敢</t>
+  </si>
+  <si>
+    <t>jung5 gam2</t>
+  </si>
+  <si>
+    <t>妥何染第件笑權</t>
+  </si>
+  <si>
+    <t>妥妥妥妥妥染染染染染何何何權妥染妥權件笑笑第何染權第件笑笑件件權染權第笑笑第何妥妥妥何權權何染染染染妥妥妥妥染染妥染染染妥妥妥妥</t>
+  </si>
+  <si>
+    <t>猛獸</t>
+  </si>
+  <si>
+    <t>maang5 sau3</t>
+  </si>
+  <si>
+    <t>友情</t>
+  </si>
+  <si>
+    <t>jau5 cing4</t>
+  </si>
+  <si>
+    <t>網站</t>
+  </si>
+  <si>
+    <t>mong5 zaam6</t>
+  </si>
+  <si>
+    <t>惘</t>
+  </si>
+  <si>
+    <t>秒我你腦買碼惘與</t>
+  </si>
+  <si>
+    <t>優雅</t>
+  </si>
+  <si>
+    <t>jau1 ngaa5</t>
+  </si>
+  <si>
+    <t>口吻</t>
+  </si>
+  <si>
+    <t>hau2 man5</t>
+  </si>
+  <si>
+    <t>過癮</t>
+  </si>
+  <si>
+    <t>gwo3 jan5</t>
+  </si>
+  <si>
+    <t>煩惱</t>
+  </si>
+  <si>
+    <t>faan4 nou5</t>
+  </si>
+  <si>
+    <t>糯米</t>
+  </si>
+  <si>
+    <t>no6 mai5</t>
+  </si>
+  <si>
+    <t>懶</t>
+  </si>
+  <si>
+    <t>laan5</t>
+  </si>
+  <si>
+    <t>奶!眼美</t>
+  </si>
+  <si>
+    <t>懶理晚武也每引遠滿朗</t>
+  </si>
+  <si>
+    <t>螞蟻|母語|魯莽|馬尾|領先|野豬|有些|勇敢|了解|敏感|挽救|軟化|猛獸|友情|儲存|偶然|冷淡|偉大|網站|優雅|温暖|風雨|展覽|小鳥|口吻|過癮|快艇|器皿|行李|牛腩|煩惱|糯米|伴舞|廟宇</t>
   </si>
 </sst>
 </file>
@@ -2685,7 +2832,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="105">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -2978,6 +3125,9 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3231,10 +3381,11 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C995"/>
+  <dimension ref="A1:C1008"/>
   <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="2" width="12.59765625" style="49" customWidth="1"/>
+    <col min="1" max="1" width="12.59765625" style="104" customWidth="1"/>
+    <col min="2" max="2" width="12.59765625" style="49" customWidth="1"/>
     <col min="3" max="3" width="12.59765625" style="50" customWidth="1"/>
     <col min="4" max="6" width="12.59765625" customWidth="1"/>
   </cols>
@@ -4872,7 +5023,7 @@
         <v>3</v>
       </c>
       <c r="B149" t="s">
-        <v>728</v>
+        <v>717</v>
       </c>
       <c r="C149" t="s">
         <v>341</v>
@@ -5166,68 +5317,68 @@
     </row>
     <row r="176" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A176" s="48">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B176" t="s">
-        <v>474</v>
+        <v>734</v>
       </c>
       <c r="C176" t="s">
-        <v>475</v>
+        <v>735</v>
       </c>
     </row>
     <row r="177" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A177" s="48">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B177" t="s">
-        <v>476</v>
+        <v>736</v>
       </c>
       <c r="C177" t="s">
-        <v>477</v>
+        <v>737</v>
       </c>
     </row>
     <row r="178" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A178" s="48">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B178" t="s">
-        <v>478</v>
+        <v>738</v>
       </c>
       <c r="C178" t="s">
-        <v>479</v>
+        <v>739</v>
       </c>
     </row>
     <row r="179" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A179" s="48">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B179" t="s">
-        <v>480</v>
+        <v>740</v>
       </c>
       <c r="C179" t="s">
-        <v>481</v>
+        <v>741</v>
       </c>
     </row>
     <row r="180" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A180" s="48">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B180" t="s">
-        <v>482</v>
+        <v>742</v>
       </c>
       <c r="C180" t="s">
-        <v>483</v>
+        <v>743</v>
       </c>
     </row>
     <row r="181" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A181" s="48">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B181" t="s">
-        <v>484</v>
+        <v>744</v>
       </c>
       <c r="C181" t="s">
-        <v>485</v>
+        <v>745</v>
       </c>
     </row>
     <row r="182" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5235,10 +5386,10 @@
         <v>4</v>
       </c>
       <c r="B182" t="s">
-        <v>486</v>
+        <v>473</v>
       </c>
       <c r="C182" t="s">
-        <v>487</v>
+        <v>474</v>
       </c>
     </row>
     <row r="183" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5246,10 +5397,10 @@
         <v>4</v>
       </c>
       <c r="B183" t="s">
-        <v>488</v>
+        <v>475</v>
       </c>
       <c r="C183" t="s">
-        <v>489</v>
+        <v>476</v>
       </c>
     </row>
     <row r="184" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5257,10 +5408,10 @@
         <v>4</v>
       </c>
       <c r="B184" t="s">
-        <v>490</v>
+        <v>477</v>
       </c>
       <c r="C184" t="s">
-        <v>491</v>
+        <v>478</v>
       </c>
     </row>
     <row r="185" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5268,10 +5419,10 @@
         <v>4</v>
       </c>
       <c r="B185" t="s">
-        <v>492</v>
+        <v>479</v>
       </c>
       <c r="C185" t="s">
-        <v>493</v>
+        <v>480</v>
       </c>
     </row>
     <row r="186" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5279,10 +5430,10 @@
         <v>4</v>
       </c>
       <c r="B186" t="s">
-        <v>494</v>
+        <v>481</v>
       </c>
       <c r="C186" t="s">
-        <v>495</v>
+        <v>482</v>
       </c>
     </row>
     <row r="187" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5290,10 +5441,10 @@
         <v>4</v>
       </c>
       <c r="B187" t="s">
-        <v>496</v>
+        <v>483</v>
       </c>
       <c r="C187" t="s">
-        <v>497</v>
+        <v>484</v>
       </c>
     </row>
     <row r="188" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5301,10 +5452,10 @@
         <v>4</v>
       </c>
       <c r="B188" t="s">
-        <v>498</v>
+        <v>485</v>
       </c>
       <c r="C188" t="s">
-        <v>499</v>
+        <v>486</v>
       </c>
     </row>
     <row r="189" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5312,10 +5463,10 @@
         <v>4</v>
       </c>
       <c r="B189" t="s">
-        <v>500</v>
+        <v>487</v>
       </c>
       <c r="C189" t="s">
-        <v>501</v>
+        <v>488</v>
       </c>
     </row>
     <row r="190" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5323,10 +5474,10 @@
         <v>4</v>
       </c>
       <c r="B190" t="s">
-        <v>502</v>
+        <v>489</v>
       </c>
       <c r="C190" t="s">
-        <v>503</v>
+        <v>490</v>
       </c>
     </row>
     <row r="191" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5334,10 +5485,10 @@
         <v>4</v>
       </c>
       <c r="B191" t="s">
-        <v>504</v>
+        <v>491</v>
       </c>
       <c r="C191" t="s">
-        <v>505</v>
+        <v>492</v>
       </c>
     </row>
     <row r="192" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5345,10 +5496,10 @@
         <v>4</v>
       </c>
       <c r="B192" t="s">
-        <v>506</v>
+        <v>493</v>
       </c>
       <c r="C192" t="s">
-        <v>507</v>
+        <v>494</v>
       </c>
     </row>
     <row r="193" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5356,10 +5507,10 @@
         <v>4</v>
       </c>
       <c r="B193" t="s">
-        <v>508</v>
+        <v>495</v>
       </c>
       <c r="C193" t="s">
-        <v>509</v>
+        <v>496</v>
       </c>
     </row>
     <row r="194" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5367,10 +5518,10 @@
         <v>4</v>
       </c>
       <c r="B194" t="s">
-        <v>510</v>
+        <v>497</v>
       </c>
       <c r="C194" t="s">
-        <v>511</v>
+        <v>498</v>
       </c>
     </row>
     <row r="195" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5378,10 +5529,10 @@
         <v>4</v>
       </c>
       <c r="B195" t="s">
-        <v>512</v>
+        <v>499</v>
       </c>
       <c r="C195" t="s">
-        <v>513</v>
+        <v>500</v>
       </c>
     </row>
     <row r="196" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5389,10 +5540,10 @@
         <v>4</v>
       </c>
       <c r="B196" t="s">
-        <v>514</v>
+        <v>501</v>
       </c>
       <c r="C196" t="s">
-        <v>515</v>
+        <v>502</v>
       </c>
     </row>
     <row r="197" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5400,10 +5551,10 @@
         <v>4</v>
       </c>
       <c r="B197" t="s">
-        <v>516</v>
+        <v>503</v>
       </c>
       <c r="C197" t="s">
-        <v>517</v>
+        <v>504</v>
       </c>
     </row>
     <row r="198" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5411,10 +5562,10 @@
         <v>4</v>
       </c>
       <c r="B198" t="s">
-        <v>536</v>
+        <v>505</v>
       </c>
       <c r="C198" t="s">
-        <v>537</v>
+        <v>506</v>
       </c>
     </row>
     <row r="199" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5422,10 +5573,10 @@
         <v>4</v>
       </c>
       <c r="B199" t="s">
-        <v>520</v>
+        <v>507</v>
       </c>
       <c r="C199" t="s">
-        <v>521</v>
+        <v>508</v>
       </c>
     </row>
     <row r="200" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5433,10 +5584,10 @@
         <v>4</v>
       </c>
       <c r="B200" t="s">
-        <v>129</v>
+        <v>509</v>
       </c>
       <c r="C200" t="s">
-        <v>522</v>
+        <v>510</v>
       </c>
     </row>
     <row r="201" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5444,10 +5595,10 @@
         <v>4</v>
       </c>
       <c r="B201" t="s">
-        <v>523</v>
+        <v>511</v>
       </c>
       <c r="C201" t="s">
-        <v>524</v>
+        <v>512</v>
       </c>
     </row>
     <row r="202" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5455,10 +5606,10 @@
         <v>4</v>
       </c>
       <c r="B202" t="s">
-        <v>525</v>
+        <v>513</v>
       </c>
       <c r="C202" t="s">
-        <v>526</v>
+        <v>514</v>
       </c>
     </row>
     <row r="203" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5466,10 +5617,10 @@
         <v>4</v>
       </c>
       <c r="B203" t="s">
-        <v>527</v>
+        <v>515</v>
       </c>
       <c r="C203" t="s">
-        <v>528</v>
+        <v>516</v>
       </c>
     </row>
     <row r="204" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5477,10 +5628,10 @@
         <v>4</v>
       </c>
       <c r="B204" t="s">
-        <v>529</v>
+        <v>535</v>
       </c>
       <c r="C204" t="s">
-        <v>530</v>
+        <v>536</v>
       </c>
     </row>
     <row r="205" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5488,10 +5639,10 @@
         <v>4</v>
       </c>
       <c r="B205" t="s">
-        <v>531</v>
+        <v>519</v>
       </c>
       <c r="C205" t="s">
-        <v>532</v>
+        <v>520</v>
       </c>
     </row>
     <row r="206" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5499,10 +5650,10 @@
         <v>4</v>
       </c>
       <c r="B206" t="s">
-        <v>533</v>
+        <v>129</v>
       </c>
       <c r="C206" t="s">
-        <v>304</v>
+        <v>521</v>
       </c>
     </row>
     <row r="207" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5510,10 +5661,10 @@
         <v>4</v>
       </c>
       <c r="B207" t="s">
-        <v>534</v>
+        <v>522</v>
       </c>
       <c r="C207" t="s">
-        <v>535</v>
+        <v>523</v>
       </c>
     </row>
     <row r="208" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5521,10 +5672,10 @@
         <v>4</v>
       </c>
       <c r="B208" t="s">
-        <v>539</v>
+        <v>524</v>
       </c>
       <c r="C208" t="s">
-        <v>540</v>
+        <v>525</v>
       </c>
     </row>
     <row r="209" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5532,21 +5683,21 @@
         <v>4</v>
       </c>
       <c r="B209" t="s">
-        <v>542</v>
+        <v>526</v>
       </c>
       <c r="C209" t="s">
-        <v>543</v>
-      </c>
-    </row>
-    <row r="210" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="210" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A210" s="48">
         <v>4</v>
       </c>
-      <c r="B210" s="103" t="s">
-        <v>731</v>
-      </c>
-      <c r="C210" s="102" t="s">
-        <v>732</v>
+      <c r="B210" t="s">
+        <v>528</v>
+      </c>
+      <c r="C210" t="s">
+        <v>529</v>
       </c>
     </row>
     <row r="211" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5554,10 +5705,10 @@
         <v>4</v>
       </c>
       <c r="B211" t="s">
-        <v>544</v>
+        <v>530</v>
       </c>
       <c r="C211" t="s">
-        <v>545</v>
+        <v>531</v>
       </c>
     </row>
     <row r="212" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5565,10 +5716,10 @@
         <v>4</v>
       </c>
       <c r="B212" t="s">
-        <v>546</v>
+        <v>532</v>
       </c>
       <c r="C212" t="s">
-        <v>547</v>
+        <v>304</v>
       </c>
     </row>
     <row r="213" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5576,10 +5727,10 @@
         <v>4</v>
       </c>
       <c r="B213" t="s">
-        <v>550</v>
+        <v>533</v>
       </c>
       <c r="C213" t="s">
-        <v>551</v>
+        <v>534</v>
       </c>
     </row>
     <row r="214" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5587,10 +5738,10 @@
         <v>4</v>
       </c>
       <c r="B214" t="s">
-        <v>552</v>
+        <v>538</v>
       </c>
       <c r="C214" t="s">
-        <v>553</v>
+        <v>539</v>
       </c>
     </row>
     <row r="215" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5598,21 +5749,21 @@
         <v>4</v>
       </c>
       <c r="B215" t="s">
-        <v>554</v>
+        <v>541</v>
       </c>
       <c r="C215" t="s">
-        <v>555</v>
-      </c>
-    </row>
-    <row r="216" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="216" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A216" s="48">
         <v>4</v>
       </c>
-      <c r="B216" t="s">
-        <v>556</v>
-      </c>
-      <c r="C216" t="s">
-        <v>557</v>
+      <c r="B216" s="103" t="s">
+        <v>720</v>
+      </c>
+      <c r="C216" s="102" t="s">
+        <v>721</v>
       </c>
     </row>
     <row r="217" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5620,10 +5771,10 @@
         <v>4</v>
       </c>
       <c r="B217" t="s">
-        <v>558</v>
+        <v>543</v>
       </c>
       <c r="C217" t="s">
-        <v>559</v>
+        <v>544</v>
       </c>
     </row>
     <row r="218" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5631,10 +5782,10 @@
         <v>4</v>
       </c>
       <c r="B218" t="s">
-        <v>560</v>
+        <v>545</v>
       </c>
       <c r="C218" t="s">
-        <v>561</v>
+        <v>546</v>
       </c>
     </row>
     <row r="219" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5642,10 +5793,10 @@
         <v>4</v>
       </c>
       <c r="B219" t="s">
-        <v>562</v>
+        <v>549</v>
       </c>
       <c r="C219" t="s">
-        <v>563</v>
+        <v>550</v>
       </c>
     </row>
     <row r="220" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5653,10 +5804,10 @@
         <v>4</v>
       </c>
       <c r="B220" t="s">
-        <v>564</v>
+        <v>551</v>
       </c>
       <c r="C220" t="s">
-        <v>565</v>
+        <v>552</v>
       </c>
     </row>
     <row r="221" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5664,10 +5815,10 @@
         <v>4</v>
       </c>
       <c r="B221" t="s">
-        <v>566</v>
+        <v>553</v>
       </c>
       <c r="C221" t="s">
-        <v>567</v>
+        <v>554</v>
       </c>
     </row>
     <row r="222" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5675,10 +5826,10 @@
         <v>4</v>
       </c>
       <c r="B222" t="s">
-        <v>568</v>
+        <v>555</v>
       </c>
       <c r="C222" t="s">
-        <v>569</v>
+        <v>556</v>
       </c>
     </row>
     <row r="223" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5686,10 +5837,10 @@
         <v>4</v>
       </c>
       <c r="B223" t="s">
-        <v>570</v>
+        <v>557</v>
       </c>
       <c r="C223" t="s">
-        <v>571</v>
+        <v>558</v>
       </c>
     </row>
     <row r="224" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5697,10 +5848,10 @@
         <v>4</v>
       </c>
       <c r="B224" t="s">
-        <v>572</v>
+        <v>559</v>
       </c>
       <c r="C224" t="s">
-        <v>573</v>
+        <v>560</v>
       </c>
     </row>
     <row r="225" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5708,10 +5859,10 @@
         <v>4</v>
       </c>
       <c r="B225" t="s">
-        <v>574</v>
+        <v>561</v>
       </c>
       <c r="C225" t="s">
-        <v>575</v>
+        <v>562</v>
       </c>
     </row>
     <row r="226" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5719,10 +5870,10 @@
         <v>4</v>
       </c>
       <c r="B226" t="s">
-        <v>576</v>
+        <v>563</v>
       </c>
       <c r="C226" t="s">
-        <v>577</v>
+        <v>564</v>
       </c>
     </row>
     <row r="227" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5730,10 +5881,10 @@
         <v>4</v>
       </c>
       <c r="B227" t="s">
-        <v>578</v>
+        <v>565</v>
       </c>
       <c r="C227" t="s">
-        <v>579</v>
+        <v>566</v>
       </c>
     </row>
     <row r="228" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5741,10 +5892,10 @@
         <v>4</v>
       </c>
       <c r="B228" t="s">
-        <v>580</v>
+        <v>567</v>
       </c>
       <c r="C228" t="s">
-        <v>581</v>
+        <v>568</v>
       </c>
     </row>
     <row r="229" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5752,10 +5903,10 @@
         <v>4</v>
       </c>
       <c r="B229" t="s">
-        <v>582</v>
+        <v>569</v>
       </c>
       <c r="C229" t="s">
-        <v>583</v>
+        <v>570</v>
       </c>
     </row>
     <row r="230" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5763,10 +5914,10 @@
         <v>4</v>
       </c>
       <c r="B230" t="s">
-        <v>584</v>
+        <v>571</v>
       </c>
       <c r="C230" t="s">
-        <v>585</v>
+        <v>572</v>
       </c>
     </row>
     <row r="231" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5774,10 +5925,10 @@
         <v>4</v>
       </c>
       <c r="B231" t="s">
-        <v>586</v>
+        <v>573</v>
       </c>
       <c r="C231" t="s">
-        <v>587</v>
+        <v>574</v>
       </c>
     </row>
     <row r="232" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5785,186 +5936,186 @@
         <v>4</v>
       </c>
       <c r="B232" t="s">
-        <v>588</v>
+        <v>575</v>
       </c>
       <c r="C232" t="s">
-        <v>589</v>
+        <v>576</v>
       </c>
     </row>
     <row r="233" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A233" s="48">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B233" t="s">
-        <v>733</v>
+        <v>577</v>
       </c>
       <c r="C233" t="s">
-        <v>734</v>
+        <v>578</v>
       </c>
     </row>
     <row r="234" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A234" s="48">
-        <v>5</v>
-      </c>
-      <c r="B234" s="93" t="s">
-        <v>602</v>
-      </c>
-      <c r="C234" s="93" t="s">
-        <v>603</v>
+        <v>4</v>
+      </c>
+      <c r="B234" t="s">
+        <v>579</v>
+      </c>
+      <c r="C234" t="s">
+        <v>580</v>
       </c>
     </row>
     <row r="235" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A235" s="48">
-        <v>5</v>
-      </c>
-      <c r="B235" s="93" t="s">
-        <v>604</v>
-      </c>
-      <c r="C235" s="93" t="s">
-        <v>605</v>
+        <v>4</v>
+      </c>
+      <c r="B235" t="s">
+        <v>581</v>
+      </c>
+      <c r="C235" t="s">
+        <v>582</v>
       </c>
     </row>
     <row r="236" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A236" s="48">
-        <v>5</v>
-      </c>
-      <c r="B236" s="95" t="s">
-        <v>675</v>
-      </c>
-      <c r="C236" s="95" t="s">
-        <v>676</v>
+        <v>4</v>
+      </c>
+      <c r="B236" t="s">
+        <v>583</v>
+      </c>
+      <c r="C236" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="237" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A237" s="48">
-        <v>5</v>
-      </c>
-      <c r="B237" s="93" t="s">
-        <v>610</v>
-      </c>
-      <c r="C237" s="93" t="s">
-        <v>611</v>
+        <v>4</v>
+      </c>
+      <c r="B237" t="s">
+        <v>585</v>
+      </c>
+      <c r="C237" t="s">
+        <v>586</v>
       </c>
     </row>
     <row r="238" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A238" s="48">
-        <v>5</v>
-      </c>
-      <c r="B238" s="95" t="s">
-        <v>677</v>
-      </c>
-      <c r="C238" s="93" t="s">
-        <v>614</v>
+        <v>4</v>
+      </c>
+      <c r="B238" t="s">
+        <v>587</v>
+      </c>
+      <c r="C238" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="239" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A239" s="48">
-        <v>5</v>
-      </c>
-      <c r="B239" s="93" t="s">
-        <v>615</v>
-      </c>
-      <c r="C239" s="93" t="s">
-        <v>616</v>
+        <v>4</v>
+      </c>
+      <c r="B239" t="s">
+        <v>747</v>
+      </c>
+      <c r="C239" t="s">
+        <v>748</v>
       </c>
     </row>
     <row r="240" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A240" s="48">
-        <v>5</v>
-      </c>
-      <c r="B240" s="93" t="s">
-        <v>612</v>
-      </c>
-      <c r="C240" s="93" t="s">
-        <v>613</v>
+        <v>4</v>
+      </c>
+      <c r="B240" t="s">
+        <v>749</v>
+      </c>
+      <c r="C240" t="s">
+        <v>750</v>
       </c>
     </row>
     <row r="241" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A241" s="48">
-        <v>5</v>
-      </c>
-      <c r="B241" s="93" t="s">
-        <v>606</v>
-      </c>
-      <c r="C241" s="93" t="s">
-        <v>607</v>
+        <v>4</v>
+      </c>
+      <c r="B241" t="s">
+        <v>751</v>
+      </c>
+      <c r="C241" t="s">
+        <v>752</v>
       </c>
     </row>
     <row r="242" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A242" s="48">
-        <v>5</v>
-      </c>
-      <c r="B242" s="93" t="s">
-        <v>608</v>
-      </c>
-      <c r="C242" s="93" t="s">
-        <v>609</v>
+        <v>4</v>
+      </c>
+      <c r="B242" t="s">
+        <v>753</v>
+      </c>
+      <c r="C242" t="s">
+        <v>754</v>
       </c>
     </row>
     <row r="243" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A243" s="48">
-        <v>5</v>
-      </c>
-      <c r="B243" s="93" t="s">
-        <v>617</v>
-      </c>
-      <c r="C243" s="93" t="s">
-        <v>618</v>
+        <v>4</v>
+      </c>
+      <c r="B243" t="s">
+        <v>755</v>
+      </c>
+      <c r="C243" t="s">
+        <v>756</v>
       </c>
     </row>
     <row r="244" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A244" s="48">
-        <v>5</v>
-      </c>
-      <c r="B244" s="95" t="s">
-        <v>671</v>
-      </c>
-      <c r="C244" s="93" t="s">
-        <v>619</v>
+        <v>4</v>
+      </c>
+      <c r="B244" t="s">
+        <v>757</v>
+      </c>
+      <c r="C244" t="s">
+        <v>758</v>
       </c>
     </row>
     <row r="245" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A245" s="48">
-        <v>5</v>
-      </c>
-      <c r="B245" s="93" t="s">
-        <v>620</v>
-      </c>
-      <c r="C245" s="93" t="s">
-        <v>621</v>
+        <v>4</v>
+      </c>
+      <c r="B245" t="s">
+        <v>759</v>
+      </c>
+      <c r="C245" t="s">
+        <v>760</v>
       </c>
     </row>
     <row r="246" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A246" s="48">
-        <v>5</v>
-      </c>
-      <c r="B246" s="93" t="s">
-        <v>626</v>
-      </c>
-      <c r="C246" s="93" t="s">
-        <v>627</v>
+        <v>4</v>
+      </c>
+      <c r="B246" t="s">
+        <v>761</v>
+      </c>
+      <c r="C246" t="s">
+        <v>762</v>
       </c>
     </row>
     <row r="247" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A247" s="48">
         <v>5</v>
       </c>
-      <c r="B247" s="93" t="s">
-        <v>628</v>
-      </c>
-      <c r="C247" s="94" t="s">
-        <v>629</v>
+      <c r="B247" t="s">
+        <v>722</v>
+      </c>
+      <c r="C247" t="s">
+        <v>723</v>
       </c>
     </row>
     <row r="248" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A248" s="48">
         <v>5</v>
       </c>
-      <c r="B248" s="95" t="s">
-        <v>632</v>
+      <c r="B248" s="93" t="s">
+        <v>599</v>
       </c>
       <c r="C248" s="93" t="s">
-        <v>633</v>
+        <v>600</v>
       </c>
     </row>
     <row r="249" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5972,21 +6123,21 @@
         <v>5</v>
       </c>
       <c r="B249" s="93" t="s">
-        <v>634</v>
+        <v>601</v>
       </c>
       <c r="C249" s="93" t="s">
-        <v>635</v>
+        <v>602</v>
       </c>
     </row>
     <row r="250" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A250" s="48">
         <v>5</v>
       </c>
-      <c r="B250" s="93" t="s">
-        <v>636</v>
-      </c>
-      <c r="C250" s="93" t="s">
-        <v>637</v>
+      <c r="B250" s="95" t="s">
+        <v>666</v>
+      </c>
+      <c r="C250" s="95" t="s">
+        <v>667</v>
       </c>
     </row>
     <row r="251" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -5994,21 +6145,21 @@
         <v>5</v>
       </c>
       <c r="B251" s="93" t="s">
-        <v>622</v>
+        <v>607</v>
       </c>
       <c r="C251" s="93" t="s">
-        <v>623</v>
+        <v>608</v>
       </c>
     </row>
     <row r="252" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A252" s="48">
         <v>5</v>
       </c>
-      <c r="B252" s="93" t="s">
-        <v>638</v>
+      <c r="B252" s="95" t="s">
+        <v>668</v>
       </c>
       <c r="C252" s="93" t="s">
-        <v>639</v>
+        <v>611</v>
       </c>
     </row>
     <row r="253" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -6016,10 +6167,10 @@
         <v>5</v>
       </c>
       <c r="B253" s="93" t="s">
-        <v>640</v>
+        <v>778</v>
       </c>
       <c r="C253" s="93" t="s">
-        <v>641</v>
+        <v>612</v>
       </c>
     </row>
     <row r="254" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -6027,10 +6178,10 @@
         <v>5</v>
       </c>
       <c r="B254" s="93" t="s">
-        <v>642</v>
+        <v>609</v>
       </c>
       <c r="C254" s="93" t="s">
-        <v>643</v>
+        <v>610</v>
       </c>
     </row>
     <row r="255" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -6038,32 +6189,32 @@
         <v>5</v>
       </c>
       <c r="B255" s="93" t="s">
-        <v>644</v>
+        <v>603</v>
       </c>
       <c r="C255" s="93" t="s">
-        <v>645</v>
+        <v>604</v>
       </c>
     </row>
     <row r="256" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A256" s="48">
         <v>5</v>
       </c>
-      <c r="B256" s="95" t="s">
-        <v>721</v>
+      <c r="B256" s="93" t="s">
+        <v>605</v>
       </c>
       <c r="C256" s="93" t="s">
-        <v>722</v>
+        <v>606</v>
       </c>
     </row>
     <row r="257" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A257" s="48">
         <v>5</v>
       </c>
-      <c r="B257" s="95" t="s">
-        <v>648</v>
+      <c r="B257" s="93" t="s">
+        <v>613</v>
       </c>
       <c r="C257" s="93" t="s">
-        <v>649</v>
+        <v>614</v>
       </c>
     </row>
     <row r="258" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -6071,43 +6222,43 @@
         <v>5</v>
       </c>
       <c r="B258" s="95" t="s">
-        <v>650</v>
+        <v>663</v>
       </c>
       <c r="C258" s="93" t="s">
-        <v>651</v>
+        <v>615</v>
       </c>
     </row>
     <row r="259" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A259" s="48">
         <v>5</v>
       </c>
-      <c r="B259" s="95" t="s">
-        <v>652</v>
+      <c r="B259" s="93" t="s">
+        <v>616</v>
       </c>
       <c r="C259" s="93" t="s">
-        <v>653</v>
+        <v>617</v>
       </c>
     </row>
     <row r="260" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A260" s="48">
         <v>5</v>
       </c>
-      <c r="B260" s="95" t="s">
-        <v>655</v>
+      <c r="B260" s="93" t="s">
+        <v>622</v>
       </c>
       <c r="C260" s="93" t="s">
-        <v>656</v>
+        <v>623</v>
       </c>
     </row>
     <row r="261" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A261" s="48">
         <v>5</v>
       </c>
-      <c r="B261" s="95" t="s">
-        <v>657</v>
-      </c>
-      <c r="C261" s="93" t="s">
-        <v>658</v>
+      <c r="B261" s="93" t="s">
+        <v>624</v>
+      </c>
+      <c r="C261" s="94" t="s">
+        <v>625</v>
       </c>
     </row>
     <row r="262" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -6115,10 +6266,10 @@
         <v>5</v>
       </c>
       <c r="B262" s="95" t="s">
-        <v>663</v>
+        <v>626</v>
       </c>
       <c r="C262" s="93" t="s">
-        <v>664</v>
+        <v>627</v>
       </c>
     </row>
     <row r="263" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -6126,21 +6277,21 @@
         <v>5</v>
       </c>
       <c r="B263" s="93" t="s">
-        <v>659</v>
+        <v>628</v>
       </c>
       <c r="C263" s="93" t="s">
-        <v>660</v>
+        <v>629</v>
       </c>
     </row>
     <row r="264" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A264" s="48">
         <v>5</v>
       </c>
-      <c r="B264" s="95" t="s">
-        <v>661</v>
+      <c r="B264" s="93" t="s">
+        <v>630</v>
       </c>
       <c r="C264" s="93" t="s">
-        <v>662</v>
+        <v>631</v>
       </c>
     </row>
     <row r="265" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -6148,43 +6299,43 @@
         <v>5</v>
       </c>
       <c r="B265" s="93" t="s">
-        <v>665</v>
+        <v>618</v>
       </c>
       <c r="C265" s="93" t="s">
-        <v>666</v>
+        <v>619</v>
       </c>
     </row>
     <row r="266" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A266" s="48">
         <v>5</v>
       </c>
-      <c r="B266" s="95" t="s">
-        <v>624</v>
+      <c r="B266" s="93" t="s">
+        <v>632</v>
       </c>
       <c r="C266" s="93" t="s">
-        <v>625</v>
+        <v>633</v>
       </c>
     </row>
     <row r="267" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A267" s="48">
         <v>5</v>
       </c>
-      <c r="B267" s="95" t="s">
-        <v>646</v>
+      <c r="B267" s="93" t="s">
+        <v>634</v>
       </c>
       <c r="C267" s="93" t="s">
-        <v>647</v>
+        <v>635</v>
       </c>
     </row>
     <row r="268" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A268" s="48">
         <v>5</v>
       </c>
-      <c r="B268" s="95" t="s">
-        <v>630</v>
+      <c r="B268" s="93" t="s">
+        <v>636</v>
       </c>
       <c r="C268" s="93" t="s">
-        <v>631</v>
+        <v>637</v>
       </c>
     </row>
     <row r="269" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -6192,87 +6343,87 @@
         <v>5</v>
       </c>
       <c r="B269" s="93" t="s">
-        <v>669</v>
+        <v>638</v>
       </c>
       <c r="C269" s="93" t="s">
-        <v>670</v>
+        <v>639</v>
       </c>
     </row>
     <row r="270" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A270" s="48">
         <v>5</v>
       </c>
-      <c r="B270" s="93" t="s">
-        <v>673</v>
+      <c r="B270" s="95" t="s">
+        <v>711</v>
       </c>
       <c r="C270" s="93" t="s">
-        <v>674</v>
+        <v>712</v>
       </c>
     </row>
     <row r="271" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A271" s="48">
         <v>5</v>
       </c>
-      <c r="B271" t="s">
-        <v>736</v>
-      </c>
-      <c r="C271" t="s">
-        <v>737</v>
+      <c r="B271" s="95" t="s">
+        <v>766</v>
+      </c>
+      <c r="C271" s="93" t="s">
+        <v>767</v>
       </c>
     </row>
     <row r="272" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A272" s="48">
         <v>5</v>
       </c>
-      <c r="B272" s="93" t="s">
-        <v>678</v>
+      <c r="B272" s="95" t="s">
+        <v>643</v>
       </c>
       <c r="C272" s="93" t="s">
-        <v>679</v>
+        <v>644</v>
       </c>
     </row>
     <row r="273" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A273" s="48">
         <v>5</v>
       </c>
-      <c r="B273" s="93" t="s">
-        <v>681</v>
+      <c r="B273" s="95" t="s">
+        <v>645</v>
       </c>
       <c r="C273" s="93" t="s">
-        <v>682</v>
+        <v>646</v>
       </c>
     </row>
     <row r="274" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A274" s="48">
         <v>5</v>
       </c>
-      <c r="B274" s="93" t="s">
-        <v>683</v>
+      <c r="B274" s="95" t="s">
+        <v>648</v>
       </c>
       <c r="C274" s="93" t="s">
-        <v>684</v>
+        <v>649</v>
       </c>
     </row>
     <row r="275" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A275" s="48">
         <v>5</v>
       </c>
-      <c r="B275" s="93" t="s">
-        <v>685</v>
+      <c r="B275" s="95" t="s">
+        <v>650</v>
       </c>
       <c r="C275" s="93" t="s">
-        <v>686</v>
+        <v>651</v>
       </c>
     </row>
     <row r="276" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A276" s="48">
         <v>5</v>
       </c>
-      <c r="B276" s="93" t="s">
-        <v>687</v>
+      <c r="B276" s="95" t="s">
+        <v>656</v>
       </c>
       <c r="C276" s="93" t="s">
-        <v>688</v>
+        <v>657</v>
       </c>
     </row>
     <row r="277" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -6280,21 +6431,21 @@
         <v>5</v>
       </c>
       <c r="B277" s="93" t="s">
-        <v>689</v>
+        <v>652</v>
       </c>
       <c r="C277" s="93" t="s">
-        <v>690</v>
+        <v>653</v>
       </c>
     </row>
     <row r="278" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A278" s="48">
         <v>5</v>
       </c>
-      <c r="B278" s="93" t="s">
-        <v>691</v>
+      <c r="B278" s="95" t="s">
+        <v>654</v>
       </c>
       <c r="C278" s="93" t="s">
-        <v>692</v>
+        <v>655</v>
       </c>
     </row>
     <row r="279" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -6302,43 +6453,43 @@
         <v>5</v>
       </c>
       <c r="B279" s="93" t="s">
-        <v>693</v>
+        <v>658</v>
       </c>
       <c r="C279" s="93" t="s">
-        <v>694</v>
+        <v>659</v>
       </c>
     </row>
     <row r="280" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A280" s="48">
         <v>5</v>
       </c>
-      <c r="B280" s="93" t="s">
-        <v>695</v>
+      <c r="B280" s="95" t="s">
+        <v>620</v>
       </c>
       <c r="C280" s="93" t="s">
-        <v>696</v>
+        <v>621</v>
       </c>
     </row>
     <row r="281" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A281" s="48">
         <v>5</v>
       </c>
-      <c r="B281" s="93" t="s">
-        <v>719</v>
+      <c r="B281" s="95" t="s">
+        <v>640</v>
       </c>
       <c r="C281" s="93" t="s">
-        <v>720</v>
+        <v>641</v>
       </c>
     </row>
     <row r="282" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A282" s="48">
         <v>5</v>
       </c>
-      <c r="B282" s="93" t="s">
-        <v>697</v>
-      </c>
-      <c r="C282" s="93" t="s">
-        <v>698</v>
+      <c r="B282" t="s">
+        <v>790</v>
+      </c>
+      <c r="C282" t="s">
+        <v>791</v>
       </c>
     </row>
     <row r="283" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -6346,10 +6497,10 @@
         <v>5</v>
       </c>
       <c r="B283" s="93" t="s">
-        <v>699</v>
+        <v>661</v>
       </c>
       <c r="C283" s="93" t="s">
-        <v>700</v>
+        <v>662</v>
       </c>
     </row>
     <row r="284" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -6357,21 +6508,21 @@
         <v>5</v>
       </c>
       <c r="B284" s="93" t="s">
-        <v>701</v>
+        <v>664</v>
       </c>
       <c r="C284" s="93" t="s">
-        <v>702</v>
+        <v>665</v>
       </c>
     </row>
     <row r="285" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A285" s="48">
         <v>5</v>
       </c>
-      <c r="B285" s="93" t="s">
-        <v>703</v>
-      </c>
-      <c r="C285" s="93" t="s">
-        <v>704</v>
+      <c r="B285" t="s">
+        <v>724</v>
+      </c>
+      <c r="C285" t="s">
+        <v>725</v>
       </c>
     </row>
     <row r="286" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -6379,10 +6530,10 @@
         <v>5</v>
       </c>
       <c r="B286" s="93" t="s">
-        <v>705</v>
+        <v>669</v>
       </c>
       <c r="C286" s="93" t="s">
-        <v>706</v>
+        <v>670</v>
       </c>
     </row>
     <row r="287" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -6390,10 +6541,10 @@
         <v>5</v>
       </c>
       <c r="B287" s="93" t="s">
-        <v>707</v>
+        <v>671</v>
       </c>
       <c r="C287" s="93" t="s">
-        <v>708</v>
+        <v>672</v>
       </c>
     </row>
     <row r="288" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -6401,10 +6552,10 @@
         <v>5</v>
       </c>
       <c r="B288" s="93" t="s">
-        <v>709</v>
+        <v>673</v>
       </c>
       <c r="C288" s="93" t="s">
-        <v>710</v>
+        <v>674</v>
       </c>
     </row>
     <row r="289" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -6412,10 +6563,10 @@
         <v>5</v>
       </c>
       <c r="B289" s="93" t="s">
-        <v>711</v>
+        <v>675</v>
       </c>
       <c r="C289" s="93" t="s">
-        <v>712</v>
+        <v>676</v>
       </c>
     </row>
     <row r="290" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -6423,10 +6574,10 @@
         <v>5</v>
       </c>
       <c r="B290" s="93" t="s">
-        <v>713</v>
+        <v>677</v>
       </c>
       <c r="C290" s="93" t="s">
-        <v>714</v>
+        <v>678</v>
       </c>
     </row>
     <row r="291" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -6434,10 +6585,10 @@
         <v>5</v>
       </c>
       <c r="B291" s="93" t="s">
-        <v>715</v>
+        <v>679</v>
       </c>
       <c r="C291" s="93" t="s">
-        <v>716</v>
+        <v>680</v>
       </c>
     </row>
     <row r="292" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -6445,40 +6596,280 @@
         <v>5</v>
       </c>
       <c r="B292" s="93" t="s">
-        <v>717</v>
+        <v>681</v>
       </c>
       <c r="C292" s="93" t="s">
-        <v>718</v>
-      </c>
-    </row>
-    <row r="293" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="294" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="295" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="296" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="297" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="298" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="299" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="300" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="301" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="302" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="303" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="304" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="305" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="306" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="307" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="308" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="309" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="310" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="311" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="312" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="313" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="314" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="315" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="316" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="317" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="318" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="319" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="320" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+        <v>682</v>
+      </c>
+    </row>
+    <row r="293" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A293" s="48">
+        <v>5</v>
+      </c>
+      <c r="B293" s="93" t="s">
+        <v>683</v>
+      </c>
+      <c r="C293" s="93" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="294" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A294" s="48">
+        <v>5</v>
+      </c>
+      <c r="B294" s="93" t="s">
+        <v>685</v>
+      </c>
+      <c r="C294" s="93" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="295" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A295" s="48">
+        <v>5</v>
+      </c>
+      <c r="B295" s="93" t="s">
+        <v>709</v>
+      </c>
+      <c r="C295" s="93" t="s">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="296" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A296" s="48">
+        <v>5</v>
+      </c>
+      <c r="B296" s="93" t="s">
+        <v>687</v>
+      </c>
+      <c r="C296" s="93" t="s">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="297" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A297" s="48">
+        <v>5</v>
+      </c>
+      <c r="B297" s="93" t="s">
+        <v>689</v>
+      </c>
+      <c r="C297" s="93" t="s">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="298" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A298" s="48">
+        <v>5</v>
+      </c>
+      <c r="B298" s="93" t="s">
+        <v>691</v>
+      </c>
+      <c r="C298" s="93" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="299" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A299" s="48">
+        <v>5</v>
+      </c>
+      <c r="B299" s="93" t="s">
+        <v>693</v>
+      </c>
+      <c r="C299" s="93" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="300" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A300" s="48">
+        <v>5</v>
+      </c>
+      <c r="B300" s="93" t="s">
+        <v>695</v>
+      </c>
+      <c r="C300" s="93" t="s">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="301" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A301" s="48">
+        <v>5</v>
+      </c>
+      <c r="B301" s="93" t="s">
+        <v>697</v>
+      </c>
+      <c r="C301" s="93" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="302" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A302" s="48">
+        <v>5</v>
+      </c>
+      <c r="B302" s="93" t="s">
+        <v>699</v>
+      </c>
+      <c r="C302" s="93" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="303" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A303" s="48">
+        <v>5</v>
+      </c>
+      <c r="B303" s="93" t="s">
+        <v>701</v>
+      </c>
+      <c r="C303" s="93" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="304" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A304" s="48">
+        <v>5</v>
+      </c>
+      <c r="B304" s="93" t="s">
+        <v>703</v>
+      </c>
+      <c r="C304" s="93" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="305" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A305" s="48">
+        <v>5</v>
+      </c>
+      <c r="B305" s="93" t="s">
+        <v>705</v>
+      </c>
+      <c r="C305" s="93" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="306" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A306" s="48">
+        <v>5</v>
+      </c>
+      <c r="B306" s="93" t="s">
+        <v>707</v>
+      </c>
+      <c r="C306" s="93" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="307" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A307" s="104">
+        <v>5</v>
+      </c>
+      <c r="B307" t="s">
+        <v>764</v>
+      </c>
+      <c r="C307" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="308" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A308" s="104">
+        <v>5</v>
+      </c>
+      <c r="B308" s="49" t="s">
+        <v>768</v>
+      </c>
+      <c r="C308" s="50" t="s">
+        <v>769</v>
+      </c>
+    </row>
+    <row r="309" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A309" s="104">
+        <v>5</v>
+      </c>
+      <c r="B309" t="s">
+        <v>772</v>
+      </c>
+      <c r="C309" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="310" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A310" s="104">
+        <v>5</v>
+      </c>
+      <c r="B310" s="49" t="s">
+        <v>774</v>
+      </c>
+      <c r="C310" s="50" t="s">
+        <v>775</v>
+      </c>
+    </row>
+    <row r="311" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A311" s="104">
+        <v>5</v>
+      </c>
+      <c r="B311" t="s">
+        <v>776</v>
+      </c>
+      <c r="C311" t="s">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="312" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A312" s="104">
+        <v>5</v>
+      </c>
+      <c r="B312" t="s">
+        <v>780</v>
+      </c>
+      <c r="C312" t="s">
+        <v>781</v>
+      </c>
+    </row>
+    <row r="313" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A313" s="104">
+        <v>5</v>
+      </c>
+      <c r="B313" t="s">
+        <v>782</v>
+      </c>
+      <c r="C313" t="s">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="314" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A314" s="104">
+        <v>5</v>
+      </c>
+      <c r="B314" t="s">
+        <v>784</v>
+      </c>
+      <c r="C314" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="315" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A315" s="104">
+        <v>5</v>
+      </c>
+      <c r="B315" t="s">
+        <v>786</v>
+      </c>
+      <c r="C315" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="316" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A316" s="104">
+        <v>5</v>
+      </c>
+      <c r="B316" s="49" t="s">
+        <v>788</v>
+      </c>
+      <c r="C316" s="50" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="317" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="318" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="319" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="320" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
     <row r="321" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
     <row r="322" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
     <row r="323" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
@@ -7154,12 +7545,25 @@
     <row r="993" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
     <row r="994" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
     <row r="995" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="996" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="1001" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="1002" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="1003" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="1004" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="1005" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="1006" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="1007" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="1008" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
   </sheetData>
-  <conditionalFormatting sqref="B176:B209 B211:B232">
-    <cfRule type="duplicateValues" dxfId="1" priority="5"/>
+  <conditionalFormatting sqref="C248:C281">
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C234:C268">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  <conditionalFormatting sqref="B182:B215 B217:B238">
+    <cfRule type="duplicateValues" dxfId="0" priority="6"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -7210,7 +7614,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>278</v>
@@ -7817,10 +8221,10 @@
         <v>3</v>
       </c>
       <c r="B22" s="51" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="C22" s="51" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
@@ -8121,10 +8525,10 @@
         <v>4</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>729</v>
+        <v>718</v>
       </c>
       <c r="C32" s="44" t="s">
-        <v>730</v>
+        <v>719</v>
       </c>
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
@@ -8145,28 +8549,28 @@
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
       <c r="E33" s="79" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="F33" s="80" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="G33" s="80" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="H33" s="80" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="I33" s="80" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="J33" s="80" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="K33" s="80" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="L33" s="81" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="M33" s="1"/>
       <c r="N33" s="1"/>
@@ -8178,28 +8582,28 @@
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
       <c r="E34" s="82" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="F34" s="23" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="G34" s="83" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="H34" s="83" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="I34" s="83" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="J34" s="83" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="K34" s="83" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="L34" s="84" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="M34" s="1"/>
       <c r="N34" s="1"/>
@@ -8211,28 +8615,28 @@
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
       <c r="E35" s="24" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="F35" s="23" t="s">
+        <v>532</v>
+      </c>
+      <c r="G35" s="23" t="s">
         <v>533</v>
       </c>
-      <c r="G35" s="23" t="s">
-        <v>534</v>
-      </c>
       <c r="H35" s="83" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="I35" s="83" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="J35" s="83" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="K35" s="83" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="L35" s="25" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="M35" s="1"/>
       <c r="N35" s="1"/>
@@ -8244,28 +8648,28 @@
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
       <c r="E36" s="24" t="s">
+        <v>532</v>
+      </c>
+      <c r="F36" s="26" t="s">
+        <v>720</v>
+      </c>
+      <c r="G36" s="23" t="s">
         <v>533</v>
       </c>
-      <c r="F36" s="26" t="s">
-        <v>731</v>
-      </c>
-      <c r="G36" s="23" t="s">
-        <v>534</v>
-      </c>
       <c r="H36" s="23" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="I36" s="83" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="J36" s="83" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="K36" s="23" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="L36" s="25" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="M36" s="1"/>
       <c r="N36" s="1"/>
@@ -8277,28 +8681,28 @@
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" s="27" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="F37" s="28" t="s">
-        <v>731</v>
+        <v>720</v>
       </c>
       <c r="G37" s="26" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="H37" s="23" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="I37" s="23" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="J37" s="23" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="K37" s="23" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="L37" s="29" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="M37" s="1"/>
       <c r="N37" s="1"/>
@@ -8310,28 +8714,28 @@
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
       <c r="E38" s="27" t="s">
-        <v>731</v>
+        <v>720</v>
       </c>
       <c r="F38" s="90" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="G38" s="26" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="H38" s="26" t="s">
-        <v>731</v>
+        <v>720</v>
       </c>
       <c r="I38" s="23" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="J38" s="23" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="K38" s="26" t="s">
-        <v>731</v>
+        <v>720</v>
       </c>
       <c r="L38" s="92" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="M38" s="1"/>
       <c r="N38" s="1"/>
@@ -8343,28 +8747,28 @@
       <c r="C39" s="1"/>
       <c r="D39" s="1"/>
       <c r="E39" s="89" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="F39" s="87" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="G39" s="90" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="H39" s="26" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="I39" s="26" t="s">
-        <v>731</v>
+        <v>720</v>
       </c>
       <c r="J39" s="26" t="s">
-        <v>731</v>
+        <v>720</v>
       </c>
       <c r="K39" s="90" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="L39" s="92" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="M39" s="1"/>
       <c r="N39" s="1"/>
@@ -8376,28 +8780,28 @@
       <c r="C40" s="1"/>
       <c r="D40" s="1"/>
       <c r="E40" s="85" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="F40" s="86" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="G40" s="86" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="H40" s="91" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="I40" s="91" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="J40" s="91" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="K40" s="86" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="L40" s="88" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="M40" s="1"/>
       <c r="N40" s="1"/>
@@ -8425,10 +8829,10 @@
         <v>5</v>
       </c>
       <c r="B42" s="51" t="s">
-        <v>667</v>
+        <v>660</v>
       </c>
       <c r="C42" s="51" t="s">
-        <v>680</v>
+        <v>770</v>
       </c>
       <c r="D42" s="1"/>
       <c r="E42" s="1"/>
@@ -8449,28 +8853,28 @@
       <c r="C43" s="1"/>
       <c r="D43" s="1"/>
       <c r="E43" s="32" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="F43" s="33" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="G43" s="33" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="H43" s="33" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="I43" s="33" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="J43" s="33" t="s">
-        <v>650</v>
+        <v>643</v>
       </c>
       <c r="K43" s="33" t="s">
-        <v>650</v>
+        <v>643</v>
       </c>
       <c r="L43" s="34" t="s">
-        <v>650</v>
+        <v>643</v>
       </c>
       <c r="M43" s="1"/>
       <c r="N43" s="1"/>
@@ -8482,28 +8886,28 @@
       <c r="C44" s="1"/>
       <c r="D44" s="1"/>
       <c r="E44" s="35" t="s">
-        <v>650</v>
+        <v>643</v>
       </c>
       <c r="F44" s="31" t="s">
-        <v>650</v>
+        <v>643</v>
       </c>
       <c r="G44" s="97" t="s">
-        <v>661</v>
+        <v>654</v>
       </c>
       <c r="H44" s="96" t="s">
-        <v>661</v>
+        <v>654</v>
       </c>
       <c r="I44" s="96" t="s">
-        <v>661</v>
+        <v>654</v>
       </c>
       <c r="J44" s="96" t="s">
-        <v>663</v>
+        <v>656</v>
       </c>
       <c r="K44" s="31" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="L44" s="36" t="s">
-        <v>650</v>
+        <v>643</v>
       </c>
       <c r="M44" s="1"/>
       <c r="N44" s="1"/>
@@ -8515,28 +8919,28 @@
       <c r="C45" s="1"/>
       <c r="D45" s="1"/>
       <c r="E45" s="35" t="s">
+        <v>642</v>
+      </c>
+      <c r="F45" s="100" t="s">
+        <v>656</v>
+      </c>
+      <c r="G45" s="51" t="s">
+        <v>650</v>
+      </c>
+      <c r="H45" s="101" t="s">
+        <v>658</v>
+      </c>
+      <c r="I45" s="101" t="s">
+        <v>658</v>
+      </c>
+      <c r="J45" s="1" t="s">
         <v>648</v>
       </c>
-      <c r="F45" s="100" t="s">
-        <v>663</v>
-      </c>
-      <c r="G45" s="51" t="s">
-        <v>657</v>
-      </c>
-      <c r="H45" s="101" t="s">
-        <v>665</v>
-      </c>
-      <c r="I45" s="101" t="s">
-        <v>665</v>
-      </c>
-      <c r="J45" s="1" t="s">
-        <v>655</v>
-      </c>
       <c r="K45" s="97" t="s">
-        <v>661</v>
+        <v>654</v>
       </c>
       <c r="L45" s="36" t="s">
-        <v>650</v>
+        <v>643</v>
       </c>
       <c r="M45" s="1"/>
       <c r="N45" s="1"/>
@@ -8548,28 +8952,28 @@
       <c r="C46" s="1"/>
       <c r="D46" s="1"/>
       <c r="E46" s="99" t="s">
-        <v>663</v>
+        <v>656</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>655</v>
+        <v>648</v>
       </c>
       <c r="G46" s="51" t="s">
-        <v>657</v>
+        <v>650</v>
       </c>
       <c r="H46" s="101" t="s">
-        <v>665</v>
+        <v>658</v>
       </c>
       <c r="I46" s="101" t="s">
-        <v>665</v>
+        <v>658</v>
       </c>
       <c r="J46" s="51" t="s">
-        <v>657</v>
+        <v>650</v>
       </c>
       <c r="K46" s="1" t="s">
-        <v>657</v>
+        <v>650</v>
       </c>
       <c r="L46" s="98" t="s">
-        <v>663</v>
+        <v>656</v>
       </c>
       <c r="M46" s="1"/>
       <c r="N46" s="1"/>
@@ -8581,28 +8985,28 @@
       <c r="C47" s="1"/>
       <c r="D47" s="1"/>
       <c r="E47" s="35" t="s">
-        <v>650</v>
+        <v>643</v>
       </c>
       <c r="F47" s="96" t="s">
-        <v>663</v>
+        <v>656</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>655</v>
+        <v>648</v>
       </c>
       <c r="H47" s="101" t="s">
-        <v>665</v>
+        <v>658</v>
       </c>
       <c r="I47" s="101" t="s">
-        <v>665</v>
+        <v>658</v>
       </c>
       <c r="J47" s="1" t="s">
-        <v>655</v>
+        <v>648</v>
       </c>
       <c r="K47" s="96" t="s">
-        <v>661</v>
+        <v>654</v>
       </c>
       <c r="L47" s="36" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="M47" s="1"/>
       <c r="N47" s="1"/>
@@ -8614,28 +9018,28 @@
       <c r="C48" s="1"/>
       <c r="D48" s="1"/>
       <c r="E48" s="35" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="F48" s="31" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="G48" s="97" t="s">
-        <v>661</v>
+        <v>654</v>
       </c>
       <c r="H48" s="97" t="s">
-        <v>663</v>
+        <v>656</v>
       </c>
       <c r="I48" s="97" t="s">
-        <v>663</v>
+        <v>656</v>
       </c>
       <c r="J48" s="96" t="s">
-        <v>661</v>
+        <v>654</v>
       </c>
       <c r="K48" s="31" t="s">
-        <v>650</v>
+        <v>643</v>
       </c>
       <c r="L48" s="36" t="s">
-        <v>650</v>
+        <v>643</v>
       </c>
       <c r="M48" s="1"/>
       <c r="N48" s="1"/>
@@ -8647,28 +9051,28 @@
       <c r="C49" s="1"/>
       <c r="D49" s="1"/>
       <c r="E49" s="35" t="s">
-        <v>650</v>
+        <v>643</v>
       </c>
       <c r="F49" s="31" t="s">
-        <v>650</v>
+        <v>643</v>
       </c>
       <c r="G49" s="31" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="H49" s="31" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="I49" s="31" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="J49" s="31" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="K49" s="31" t="s">
-        <v>650</v>
+        <v>643</v>
       </c>
       <c r="L49" s="36" t="s">
-        <v>650</v>
+        <v>643</v>
       </c>
       <c r="M49" s="1"/>
       <c r="N49" s="1"/>
@@ -8680,28 +9084,28 @@
       <c r="C50" s="1"/>
       <c r="D50" s="1"/>
       <c r="E50" s="37" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="F50" s="38" t="s">
-        <v>650</v>
+        <v>643</v>
       </c>
       <c r="G50" s="38" t="s">
-        <v>650</v>
+        <v>643</v>
       </c>
       <c r="H50" s="38" t="s">
-        <v>650</v>
+        <v>643</v>
       </c>
       <c r="I50" s="38" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="J50" s="38" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="K50" s="38" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="L50" s="39" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="M50" s="1"/>
       <c r="N50" s="1"/>
@@ -12746,7 +13150,7 @@
     <col min="1" max="1" width="7.3984375" customWidth="1"/>
     <col min="2" max="2" width="17.59765625" customWidth="1"/>
     <col min="3" max="3" width="18.86328125" customWidth="1"/>
-    <col min="4" max="4" width="47.1328125" customWidth="1"/>
+    <col min="4" max="4" width="52.53125" customWidth="1"/>
     <col min="5" max="8" width="18.86328125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -12814,7 +13218,7 @@
         <v>11</v>
       </c>
       <c r="D4" s="51" t="s">
-        <v>741</v>
+        <v>728</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
@@ -12868,7 +13272,7 @@
         <v>11</v>
       </c>
       <c r="D7" s="51" t="s">
-        <v>740</v>
+        <v>727</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -12970,13 +13374,13 @@
         <v>1</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
@@ -12988,13 +13392,13 @@
         <v>1</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
@@ -13102,7 +13506,7 @@
         <v>11</v>
       </c>
       <c r="D20" s="51" t="s">
-        <v>742</v>
+        <v>729</v>
       </c>
       <c r="E20" s="48"/>
       <c r="F20" s="1"/>
@@ -13186,13 +13590,13 @@
         <v>2</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="E25" s="48"/>
       <c r="F25" s="1"/>
@@ -13204,13 +13608,13 @@
         <v>2</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="E26" s="48"/>
       <c r="F26" s="1"/>
@@ -13246,7 +13650,7 @@
         <v>24</v>
       </c>
       <c r="D28" s="51" t="s">
-        <v>726</v>
+        <v>715</v>
       </c>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
@@ -13318,7 +13722,7 @@
         <v>11</v>
       </c>
       <c r="D32" s="51" t="s">
-        <v>743</v>
+        <v>730</v>
       </c>
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
@@ -13390,7 +13794,7 @@
         <v>18</v>
       </c>
       <c r="D36" s="44" t="s">
-        <v>727</v>
+        <v>716</v>
       </c>
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
@@ -13398,15 +13802,17 @@
       <c r="H36" s="1"/>
     </row>
     <row r="37" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A37" s="3"/>
+      <c r="A37" s="3">
+        <v>3</v>
+      </c>
       <c r="B37" s="3" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D37" s="51" t="s">
-        <v>600</v>
+        <v>733</v>
       </c>
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>
@@ -13418,13 +13824,13 @@
         <v>3</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
@@ -13460,7 +13866,7 @@
         <v>24</v>
       </c>
       <c r="D40" s="51" t="s">
-        <v>473</v>
+        <v>746</v>
       </c>
       <c r="E40" s="1"/>
       <c r="F40" s="1"/>
@@ -13532,7 +13938,7 @@
         <v>11</v>
       </c>
       <c r="D44" s="51" t="s">
-        <v>744</v>
+        <v>731</v>
       </c>
       <c r="E44" s="1"/>
       <c r="F44" s="1"/>
@@ -13550,7 +13956,7 @@
         <v>13</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
@@ -13568,7 +13974,7 @@
         <v>15</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
@@ -13586,7 +13992,7 @@
         <v>17</v>
       </c>
       <c r="D47" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
@@ -13604,7 +14010,7 @@
         <v>18</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="E48" s="1"/>
       <c r="F48" s="1"/>
@@ -13612,15 +14018,17 @@
       <c r="H48" s="1"/>
     </row>
     <row r="49" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A49" s="3"/>
+      <c r="A49" s="3">
+        <v>4</v>
+      </c>
       <c r="B49" s="3" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="C49" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="E49" s="1"/>
       <c r="F49" s="1"/>
@@ -13632,13 +14040,13 @@
         <v>4</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="C50" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D50" s="51" t="s">
-        <v>739</v>
+        <v>726</v>
       </c>
       <c r="E50" s="1"/>
       <c r="F50" s="1"/>
@@ -13656,14 +14064,14 @@
         <v>21</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="E51" s="1"/>
       <c r="F51" s="1"/>
       <c r="G51" s="1"/>
       <c r="H51" s="1"/>
     </row>
-    <row r="52" spans="1:8" ht="30.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:8" ht="41.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A52" s="3">
         <v>4</v>
       </c>
@@ -13674,7 +14082,7 @@
         <v>24</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>590</v>
+        <v>763</v>
       </c>
       <c r="E52" s="1"/>
       <c r="F52" s="1"/>
@@ -13746,7 +14154,7 @@
         <v>11</v>
       </c>
       <c r="D56" s="51" t="s">
-        <v>745</v>
+        <v>732</v>
       </c>
       <c r="E56" s="1"/>
       <c r="F56" s="1"/>
@@ -13764,7 +14172,7 @@
         <v>13</v>
       </c>
       <c r="D57" s="51" t="s">
-        <v>735</v>
+        <v>779</v>
       </c>
       <c r="E57" s="1"/>
       <c r="F57" s="1"/>
@@ -13782,7 +14190,7 @@
         <v>15</v>
       </c>
       <c r="D58" s="51" t="s">
-        <v>672</v>
+        <v>793</v>
       </c>
       <c r="E58" s="1"/>
       <c r="F58" s="1"/>
@@ -13800,7 +14208,7 @@
         <v>17</v>
       </c>
       <c r="D59" s="51" t="s">
-        <v>654</v>
+        <v>647</v>
       </c>
       <c r="E59" s="1"/>
       <c r="F59" s="1"/>
@@ -13818,7 +14226,7 @@
         <v>18</v>
       </c>
       <c r="D60" s="51" t="s">
-        <v>723</v>
+        <v>713</v>
       </c>
       <c r="E60" s="1"/>
       <c r="F60" s="1"/>
@@ -13826,15 +14234,17 @@
       <c r="H60" s="1"/>
     </row>
     <row r="61" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A61" s="3"/>
+      <c r="A61" s="3">
+        <v>5</v>
+      </c>
       <c r="B61" s="3" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="C61" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D61" s="51" t="s">
-        <v>725</v>
+        <v>714</v>
       </c>
       <c r="E61" s="1"/>
       <c r="F61" s="1"/>
@@ -13846,13 +14256,13 @@
         <v>5</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="C62" s="3" t="s">
         <v>21</v>
       </c>
       <c r="D62" s="51" t="s">
-        <v>724</v>
+        <v>771</v>
       </c>
       <c r="E62" s="1"/>
       <c r="F62" s="1"/>
@@ -13870,7 +14280,7 @@
         <v>21</v>
       </c>
       <c r="D63" s="51" t="s">
-        <v>668</v>
+        <v>792</v>
       </c>
       <c r="E63" s="1"/>
       <c r="F63" s="1"/>
@@ -13888,7 +14298,7 @@
         <v>24</v>
       </c>
       <c r="D64" s="51" t="s">
-        <v>738</v>
+        <v>794</v>
       </c>
       <c r="E64" s="1"/>
       <c r="F64" s="1"/>

</xml_diff>